<commit_message>
Expand mega job list to 63 roles - add EY, KPMG, PwC, NTT DATA supply chain planning jobs
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job_listings_mega.xlsx
+++ b/job_listings_mega.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3529,168 +3529,722 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
+          <t>SC Tech - OMP Planning Mgr ⭐⭐
+(Location OPEN)</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>USA (Remote-Flexible)</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K54" s="9" t="inlineStr">
+        <is>
+          <t>OMP in job title! · Location OPEN · S&amp;OP/IBP transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>SAP - SC Planning IBP PPDS Mgr ⭐
+(Location OPEN)</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>Chicago, IL (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>$141K–$258K 💰</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I55" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>5+ yrs SAP IBP/APO · S&amp;OP/IBP · $141K–$258K · Location OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>SC Health - Perf Improvement Mgr</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>Nashville, TN (On-site)</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>On-site · FT</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>✅ GOOD</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I56" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J56" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K56" s="9" t="inlineStr">
+        <is>
+          <t>30 o9 alumni · SC performance improvement consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>SC &amp; Ops Senior Consultant</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>Nashville, TN (On-site)</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>On-site · FT</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>✅ GOOD</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I57" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J57" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K57" s="9" t="inlineStr">
+        <is>
+          <t>30 o9 alumni · Be an early applicant! · SC &amp; Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="40" customHeight="1">
+      <c r="A58" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>SC Procurement Mgr – Multiple
+(Positions 1696063)</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>Atlanta, GA (On-site)</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>On-site · FT</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>✅ GOOD</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I58" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K58" s="9" t="inlineStr">
+        <is>
+          <t>30 o9 alumni · Multiple positions open · SC procurement &amp; planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>Manager, SAP Supply Chain (IBP)</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>Multiple US</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I59" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K59" s="9" t="inlineStr">
+        <is>
+          <t>SAP IBP implementation · SC planning background · 6000+ SAP consultants</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>SAP SC - IBP Solution Architect
+Sr. Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>New York, NY + 11 locations</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>$130K–$256K 💰</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I60" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J60" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K60" s="9" t="inlineStr">
+        <is>
+          <t>IBP Demand/Supply/Inventory/S&amp;OP · Solution Architect Sr Mgr · $130K–$256K!</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>SAP IBP/TM/PP Senior Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>Atlanta, GA (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>$130K–$256K 💰</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I61" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J61" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K61" s="9" t="inlineStr">
+        <is>
+          <t>SAP IBP + Transportation Mgmt + PP · Senior Manager level</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>SAP IBP Senior Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr">
+        <is>
+          <t>Dallas, TX (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>$130K–$256K 💰</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H62" s="9" t="inlineStr">
+        <is>
+          <t>Big 4</t>
+        </is>
+      </c>
+      <c r="I62" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J62" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K62" s="9" t="inlineStr">
+        <is>
+          <t>SAP IBP focused · $130K–$256K · Dallas location</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="40" customHeight="1">
+      <c r="A63" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>o9 Consulting Manager ⭐⭐</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>NTT DATA North America</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>Georgia (Remote)</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>Remote · FT</t>
+        </is>
+      </c>
+      <c r="F63" s="13" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="I63" s="14" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J63" s="13" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K63" s="13" t="inlineStr">
+        <is>
+          <t>o9 IN TITLE! · Remote · NTT DATA SC Consulting · 13 alumni · Be early applicant</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="40" customHeight="1">
+      <c r="A64" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" s="9" t="inlineStr">
+        <is>
           <t>SC Planning Solutions Consultant ⭐⭐
 (BY/Kinaxis/OMP/O9)</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>Accenture</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr">
+      <c r="D64" s="9" t="inlineStr">
         <is>
           <t>St. Louis, MO / US</t>
         </is>
       </c>
-      <c r="E54" s="9" t="inlineStr">
+      <c r="E64" s="9" t="inlineStr">
         <is>
           <t>Hybrid · FT</t>
         </is>
       </c>
-      <c r="F54" s="9" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="F64" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>⭐⭐ PERFECT</t>
         </is>
       </c>
-      <c r="H54" s="9" t="inlineStr">
+      <c r="H64" s="9" t="inlineStr">
         <is>
           <t>Big 4</t>
         </is>
       </c>
-      <c r="I54" s="10" t="inlineStr">
-        <is>
-          <t>View Job →</t>
-        </is>
-      </c>
-      <c r="J54" s="9" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="K54" s="9" t="inlineStr">
+      <c r="I64" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J64" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K64" s="9" t="inlineStr">
         <is>
           <t>BY, Kinaxis, OMP, O9 all in title! · Veterans preferred</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="40" customHeight="1">
-      <c r="A55" s="24" t="n">
-        <v>52</v>
-      </c>
-      <c r="B55" s="25" t="inlineStr">
+    <row r="65" ht="40" customHeight="1">
+      <c r="A65" s="24" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" s="25" t="inlineStr">
         <is>
           <t>O9 Supply Chain Technical Lead</t>
         </is>
       </c>
-      <c r="C55" s="25" t="inlineStr">
+      <c r="C65" s="25" t="inlineStr">
         <is>
           <t>Net2Source Inc.</t>
         </is>
       </c>
-      <c r="D55" s="25" t="inlineStr">
+      <c r="D65" s="25" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
       </c>
-      <c r="E55" s="25" t="inlineStr">
+      <c r="E65" s="25" t="inlineStr">
         <is>
           <t>On-site · Contract</t>
         </is>
       </c>
-      <c r="F55" s="25" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="F65" s="25" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
         <is>
           <t>⭐⭐ PERFECT</t>
         </is>
       </c>
-      <c r="H55" s="25" t="inlineStr">
+      <c r="H65" s="25" t="inlineStr">
         <is>
           <t>Staffing</t>
         </is>
       </c>
-      <c r="I55" s="26" t="inlineStr">
-        <is>
-          <t>View Job →</t>
-        </is>
-      </c>
-      <c r="J55" s="25" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="K55" s="25" t="inlineStr">
+      <c r="I65" s="26" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J65" s="25" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K65" s="25" t="inlineStr">
         <is>
           <t>7+ yrs o9 · Demand/Supply/S&amp;OP · Technical + functional</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="40" customHeight="1">
-      <c r="A56" s="12" t="n">
-        <v>53</v>
-      </c>
-      <c r="B56" s="13" t="inlineStr">
+    <row r="66" ht="40" customHeight="1">
+      <c r="A66" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>Consultant – SC &amp; Ops</t>
         </is>
       </c>
-      <c r="C56" s="13" t="inlineStr">
+      <c r="C66" s="13" t="inlineStr">
         <is>
           <t>Rios Partners</t>
         </is>
       </c>
-      <c r="D56" s="13" t="inlineStr">
+      <c r="D66" s="13" t="inlineStr">
         <is>
           <t>Arlington, VA</t>
         </is>
       </c>
-      <c r="E56" s="13" t="inlineStr">
+      <c r="E66" s="13" t="inlineStr">
         <is>
           <t>On-site · FT</t>
         </is>
       </c>
-      <c r="F56" s="13" t="inlineStr">
+      <c r="F66" s="13" t="inlineStr">
         <is>
           <t>$110K–$130K 💰</t>
         </is>
       </c>
-      <c r="G56" s="11" t="inlineStr">
+      <c r="G66" s="11" t="inlineStr">
         <is>
           <t>✅ GOOD</t>
         </is>
       </c>
-      <c r="H56" s="13" t="inlineStr">
+      <c r="H66" s="13" t="inlineStr">
         <is>
           <t>Consulting</t>
         </is>
       </c>
-      <c r="I56" s="14" t="inlineStr">
-        <is>
-          <t>View Job →</t>
-        </is>
-      </c>
-      <c r="J56" s="13" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="K56" s="13" t="inlineStr">
+      <c r="I66" s="14" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="J66" s="13" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K66" s="13" t="inlineStr">
         <is>
           <t>SC consulting boutique · $110K–$130K base</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="27" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="27" t="inlineStr">
         <is>
           <t>🟡 o9 Direct   🔵 Big 4 / Consulting   🟠 SC Vendor   ⚪ Industry   ⭐⭐PERFECT = o9/OMP in job title   ⭐HIGH = SC planning tech   ✅GOOD = SC consulting</t>
         </is>
@@ -3698,8 +4252,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A58:K58"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A68:K68"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId1"/>
@@ -3754,6 +4308,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3765,7 +4329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4602,96 +5166,248 @@
       </c>
       <c r="B19" s="34" t="inlineStr">
         <is>
+          <t>SC Tech - OMP Planning Mgr ⭐⭐
+(Location OPEN)</t>
+        </is>
+      </c>
+      <c r="C19" s="34" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D19" s="34" t="inlineStr">
+        <is>
+          <t>USA (Remote-Flexible)</t>
+        </is>
+      </c>
+      <c r="E19" s="34" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H19" s="35" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I19" s="34" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J19" s="34" t="inlineStr">
+        <is>
+          <t>OMP in job title! · Location OPEN · S&amp;OP/IBP transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="30" t="n">
+        <v>57</v>
+      </c>
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>SAP SC - IBP Solution Architect
+Sr. Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="D20" s="31" t="inlineStr">
+        <is>
+          <t>New York, NY + 11 locations</t>
+        </is>
+      </c>
+      <c r="E20" s="31" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F20" s="31" t="inlineStr">
+        <is>
+          <t>$130K–$256K 💰</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H20" s="32" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I20" s="31" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J20" s="31" t="inlineStr">
+        <is>
+          <t>IBP Demand/Supply/Inventory/S&amp;OP · Solution Architect Sr Mgr · $130K–$256K!</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="33" t="n">
+        <v>60</v>
+      </c>
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>o9 Consulting Manager ⭐⭐</t>
+        </is>
+      </c>
+      <c r="C21" s="34" t="inlineStr">
+        <is>
+          <t>NTT DATA North America</t>
+        </is>
+      </c>
+      <c r="D21" s="34" t="inlineStr">
+        <is>
+          <t>Georgia (Remote)</t>
+        </is>
+      </c>
+      <c r="E21" s="34" t="inlineStr">
+        <is>
+          <t>Remote · FT</t>
+        </is>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H21" s="35" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I21" s="34" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J21" s="34" t="inlineStr">
+        <is>
+          <t>o9 IN TITLE! · Remote · NTT DATA SC Consulting · 13 alumni · Be early applicant</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="30" t="n">
+        <v>61</v>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
           <t>SC Planning Solutions Consultant ⭐⭐
 (BY/Kinaxis/OMP/O9)</t>
         </is>
       </c>
-      <c r="C19" s="34" t="inlineStr">
+      <c r="C22" s="31" t="inlineStr">
         <is>
           <t>Accenture</t>
         </is>
       </c>
-      <c r="D19" s="34" t="inlineStr">
+      <c r="D22" s="31" t="inlineStr">
         <is>
           <t>St. Louis, MO / US</t>
         </is>
       </c>
-      <c r="E19" s="34" t="inlineStr">
+      <c r="E22" s="31" t="inlineStr">
         <is>
           <t>Hybrid · FT</t>
         </is>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="F22" s="31" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>⭐⭐ PERFECT</t>
         </is>
       </c>
-      <c r="H19" s="35" t="inlineStr">
-        <is>
-          <t>View Job →</t>
-        </is>
-      </c>
-      <c r="I19" s="34" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="J19" s="34" t="inlineStr">
+      <c r="H22" s="32" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I22" s="31" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J22" s="31" t="inlineStr">
         <is>
           <t>BY, Kinaxis, OMP, O9 all in title! · Veterans preferred</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="30" t="n">
-        <v>52</v>
-      </c>
-      <c r="B20" s="31" t="inlineStr">
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="33" t="n">
+        <v>62</v>
+      </c>
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>O9 Supply Chain Technical Lead</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C23" s="34" t="inlineStr">
         <is>
           <t>Net2Source Inc.</t>
         </is>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D23" s="34" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
       </c>
-      <c r="E20" s="31" t="inlineStr">
+      <c r="E23" s="34" t="inlineStr">
         <is>
           <t>On-site · Contract</t>
         </is>
       </c>
-      <c r="F20" s="31" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>⭐⭐ PERFECT</t>
         </is>
       </c>
-      <c r="H20" s="32" t="inlineStr">
-        <is>
-          <t>View Job →</t>
-        </is>
-      </c>
-      <c r="I20" s="31" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="J20" s="31" t="inlineStr">
+      <c r="H23" s="35" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I23" s="34" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J23" s="34" t="inlineStr">
         <is>
           <t>7+ yrs o9 · Demand/Supply/S&amp;OP · Technical + functional</t>
         </is>
@@ -4719,6 +5435,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4730,7 +5449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6019,96 +6738,600 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
+          <t>SC Tech - OMP Planning Mgr ⭐⭐
+(Location OPEN)</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>USA (Remote-Flexible)</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>OMP in job title! · Location OPEN · S&amp;OP/IBP transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="21" t="n">
+        <v>52</v>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>SAP - SC Planning IBP PPDS Mgr ⭐
+(Location OPEN)</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Chicago, IL (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>$141K–$258K 💰</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H29" s="36" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I29" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J29" s="22" t="inlineStr">
+        <is>
+          <t>5+ yrs SAP IBP/APO · S&amp;OP/IBP · $141K–$258K · Location OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>SC Health - Perf Improvement Mgr</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Nashville, TN (On-site)</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>On-site · FT</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>✅ GOOD</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>30 o9 alumni · SC performance improvement consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="21" t="n">
+        <v>54</v>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>SC &amp; Ops Senior Consultant</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Nashville, TN (On-site)</t>
+        </is>
+      </c>
+      <c r="E31" s="22" t="inlineStr">
+        <is>
+          <t>On-site · FT</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>✅ GOOD</t>
+        </is>
+      </c>
+      <c r="H31" s="36" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I31" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J31" s="22" t="inlineStr">
+        <is>
+          <t>30 o9 alumni · Be an early applicant! · SC &amp; Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>SC Procurement Mgr – Multiple
+(Positions 1696063)</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Atlanta, GA (On-site)</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>On-site · FT</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>✅ GOOD</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>30 o9 alumni · Multiple positions open · SC procurement &amp; planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="21" t="n">
+        <v>56</v>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>Manager, SAP Supply Chain (IBP)</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Multiple US</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H33" s="36" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I33" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J33" s="22" t="inlineStr">
+        <is>
+          <t>SAP IBP implementation · SC planning background · 6000+ SAP consultants</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>SAP SC - IBP Solution Architect
+Sr. Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>New York, NY + 11 locations</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>$130K–$256K 💰</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>IBP Demand/Supply/Inventory/S&amp;OP · Solution Architect Sr Mgr · $130K–$256K!</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="21" t="n">
+        <v>58</v>
+      </c>
+      <c r="B35" s="22" t="inlineStr">
+        <is>
+          <t>SAP IBP/TM/PP Senior Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>Atlanta, GA (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E35" s="22" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F35" s="22" t="inlineStr">
+        <is>
+          <t>$130K–$256K 💰</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H35" s="36" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I35" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J35" s="22" t="inlineStr">
+        <is>
+          <t>SAP IBP + Transportation Mgmt + PP · Senior Manager level</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>SAP IBP Senior Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Dallas, TX (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>Hybrid · FT</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>$130K–$256K 💰</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>⭐ HIGH</t>
+        </is>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J36" s="9" t="inlineStr">
+        <is>
+          <t>SAP IBP focused · $130K–$256K · Dallas location</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" s="21" t="n">
+        <v>60</v>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>o9 Consulting Manager ⭐⭐</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t>NTT DATA North America</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>Georgia (Remote)</t>
+        </is>
+      </c>
+      <c r="E37" s="22" t="inlineStr">
+        <is>
+          <t>Remote · FT</t>
+        </is>
+      </c>
+      <c r="F37" s="22" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐ PERFECT</t>
+        </is>
+      </c>
+      <c r="H37" s="36" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I37" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J37" s="22" t="inlineStr">
+        <is>
+          <t>o9 IN TITLE! · Remote · NTT DATA SC Consulting · 13 alumni · Be early applicant</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
           <t>SC Planning Solutions Consultant ⭐⭐
 (BY/Kinaxis/OMP/O9)</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Accenture</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D38" s="9" t="inlineStr">
         <is>
           <t>St. Louis, MO / US</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Hybrid · FT</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>Not listed</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>⭐⭐ PERFECT</t>
         </is>
       </c>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>View Job →</t>
-        </is>
-      </c>
-      <c r="I28" s="9" t="inlineStr">
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I38" s="9" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="J28" s="9" t="inlineStr">
+      <c r="J38" s="9" t="inlineStr">
         <is>
           <t>BY, Kinaxis, OMP, O9 all in title! · Veterans preferred</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="42" customHeight="1">
-      <c r="A29" s="21" t="n">
-        <v>53</v>
-      </c>
-      <c r="B29" s="22" t="inlineStr">
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" s="21" t="n">
+        <v>63</v>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>Consultant – SC &amp; Ops</t>
         </is>
       </c>
-      <c r="C29" s="22" t="inlineStr">
+      <c r="C39" s="22" t="inlineStr">
         <is>
           <t>Rios Partners</t>
         </is>
       </c>
-      <c r="D29" s="22" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>Arlington, VA</t>
         </is>
       </c>
-      <c r="E29" s="22" t="inlineStr">
+      <c r="E39" s="22" t="inlineStr">
         <is>
           <t>On-site · FT</t>
         </is>
       </c>
-      <c r="F29" s="22" t="inlineStr">
+      <c r="F39" s="22" t="inlineStr">
         <is>
           <t>$110K–$130K 💰</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>✅ GOOD</t>
         </is>
       </c>
-      <c r="H29" s="36" t="inlineStr">
-        <is>
-          <t>View Job →</t>
-        </is>
-      </c>
-      <c r="I29" s="22" t="inlineStr">
+      <c r="H39" s="36" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I39" s="22" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="J29" s="22" t="inlineStr">
+      <c r="J39" s="22" t="inlineStr">
         <is>
           <t>SC consulting boutique · $110K–$130K base</t>
         </is>
@@ -6145,6 +7368,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6685,7 +7918,7 @@
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="21" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="B13" s="22" t="inlineStr">
         <is>

</xml_diff>